<commit_message>
docs: S03 acta + TC-064 Parcial + RNF 1.0.2
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/fase2/Evidencias Proyecto/Evidencias de Documentacion/05_Documento_de_Diseno/03_RNF/DPAY3_Catalogo_RNF_v1.0.xlsx
+++ b/fase2/Evidencias Proyecto/Evidencias de Documentacion/05_Documento_de_Diseno/03_RNF/DPAY3_Catalogo_RNF_v1.0.xlsx
@@ -864,7 +864,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>1.0.1</t>
+          <t>1.0.2</t>
         </is>
       </c>
       <c r="D9" s="37" t="n"/>
@@ -878,7 +878,7 @@
       </c>
       <c r="C10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="D10" s="37" t="n"/>
@@ -2073,7 +2073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S36"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="11" customWidth="1" style="33" min="1" max="1"/>
@@ -2111,7 +2111,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="33">
       <c r="A4" s="18" t="inlineStr">
         <is>
@@ -2374,12 +2373,12 @@
       </c>
       <c r="N6" s="27" t="inlineStr">
         <is>
-          <t>hu06Tuu.test.ts + operación en producción (Diego)</t>
+          <t>COD-08-HU06-tuu-kozen/capturas/TC-RG-01*; 07_Plan_de_Pruebas/05_Evidencias_por_sprint/Sprint_03/capturas_20261013/; jest-hu06Tuu-factory-deteccion-output-20261011.txt</t>
         </is>
       </c>
       <c r="O6" s="26" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="P6" s="27" t="inlineStr">
@@ -2399,7 +2398,7 @@
       </c>
       <c r="S6" s="27" t="inlineStr">
         <is>
-          <t>El DAS describe Intent TUU en Kozen (CU-03, restricción Hardware TUU) sin métrica de 2 s. El umbral es del DoD. Línea base D-PAY 2.0 en producción, operada por Diego. «Bloqueado» solo para la regresión manual del equipo QA (sin terminal).</t>
+          <t>Parcial 13/10/2026: Diego Madrid, Kozen P8 Neo. Débito $2.000 aprobado; crédito $5.000 cancelado (no declined emisor). Falta crédito aprobado. Jest 17/17 (11/10).</t>
         </is>
       </c>
     </row>
@@ -4007,12 +4006,12 @@
       </c>
       <c r="N23" s="27" t="inlineStr">
         <is>
-          <t>abiFilters armeabi-v7a · operación Diego</t>
+          <t>COD-08-HU06-tuu-kozen/capturas/TC-RG-01*; 07_Plan_de_Pruebas/05_Evidencias_por_sprint/Sprint_03/capturas_20261013/; jest-hu06Tuu-factory-deteccion-output-20261011.txt</t>
         </is>
       </c>
       <c r="O23" s="26" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="P23" s="27" t="inlineStr">
@@ -4032,7 +4031,7 @@
       </c>
       <c r="S23" s="27" t="inlineStr">
         <is>
-          <t>Alineado con el DAS (Kozen + TUU). Producción D-PAY 2.0 (Diego). Bloqueo solo de la regresión manual en QA Capstone.</t>
+          <t>Parcial 13/10/2026: Diego Madrid, Kozen P8 Neo. Débito $2.000 aprobado; crédito $5.000 cancelado (no declined emisor). Falta crédito aprobado. Jest 17/17 (11/10).</t>
         </is>
       </c>
     </row>
@@ -6343,7 +6342,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="33">
       <c r="A4" s="18" t="inlineStr">
         <is>
@@ -7945,7 +7943,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
         <is>
@@ -8383,7 +8380,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(fase2): alinea S03 cerrada y tipografia en evidencias APT
Publica Word/md/txt auditados (guion, ver Seccion, Retro S03 15/10, Goal Parcial). Conserva planillas Excel y DAS renombrado.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/fase2/Evidencias Proyecto/Evidencias de Documentacion/05_Documento_de_Diseno/03_RNF/DPAY3_Catalogo_RNF_v1.0.xlsx
+++ b/fase2/Evidencias Proyecto/Evidencias de Documentacion/05_Documento_de_Diseno/03_RNF/DPAY3_Catalogo_RNF_v1.0.xlsx
@@ -801,7 +801,7 @@
     <row r="2">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>D-PAY 3.0 — Catálogo de Requerimientos No Funcionales</t>
+          <t>D-PAY 3.0 - Catálogo de Requerimientos No Funcionales</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="C6" s="36" t="inlineStr">
         <is>
-          <t>D-PAY 3.0 — POS móvil multi-pasarela (DTemite)</t>
+          <t>D-PAY 3.0 - POS móvil multi-pasarela (DTemite)</t>
         </is>
       </c>
       <c r="D6" s="37" t="n"/>
@@ -836,7 +836,7 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>Capstone PTY4614 / APT122 — Duoc UC 2026-2</t>
+          <t>Capstone PTY4614 / APT122 - Duoc UC 2026-2</t>
         </is>
       </c>
       <c r="D7" s="37" t="n"/>
@@ -850,7 +850,7 @@
       </c>
       <c r="C8" s="36" t="inlineStr">
         <is>
-          <t>Catálogo RNF (anexo del DAS §Metas y §Escenarios)</t>
+          <t>Catálogo RNF (anexo del DAS ver Seccion Metas y ver Seccion Escenarios)</t>
         </is>
       </c>
       <c r="D8" s="37" t="n"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>1.0.1</t>
+          <t>1.0.2</t>
         </is>
       </c>
       <c r="D9" s="37" t="n"/>
@@ -878,7 +878,7 @@
       </c>
       <c r="C10" s="36" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="D10" s="37" t="n"/>
@@ -2100,7 +2100,7 @@
     <row r="1" ht="30" customHeight="1" s="33">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>Catálogo RNF — D-PAY 3.0</t>
+          <t>Catálogo RNF - D-PAY 3.0</t>
         </is>
       </c>
     </row>
@@ -2374,12 +2374,12 @@
       </c>
       <c r="N6" s="27" t="inlineStr">
         <is>
-          <t>hu06Tuu.test.ts + operación en producción (Diego)</t>
+          <t>COD-08-HU06-tuu-kozen/capturas/TC-RG-01*; 07_Plan_de_Pruebas/05_Evidencias_por_sprint/Sprint_03/capturas_20261013/; jest-hu06Tuu-factory-deteccion-output-20261011.txt</t>
         </is>
       </c>
       <c r="O6" s="26" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="P6" s="27" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="S6" s="27" t="inlineStr">
         <is>
-          <t>El DAS describe Intent TUU en Kozen (CU-03, restricción Hardware TUU) sin métrica de 2 s. El umbral es del DoD. Línea base D-PAY 2.0 en producción, operada por Diego. «Bloqueado» solo para la regresión manual del equipo QA (sin terminal).</t>
+          <t>Parcial 13/10/2026: Diego Madrid, Kozen P8 Neo. Débito $2.000 aprobado; crédito $5.000 cancelado (no declined emisor). Falta crédito aprobado. Jest 17/17 (11/10).</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="N8" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O8" s="26" t="inlineStr">
@@ -3230,12 +3230,12 @@
       </c>
       <c r="M15" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N15" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O15" s="26" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="N20" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O20" s="26" t="inlineStr">
@@ -3808,12 +3808,12 @@
       </c>
       <c r="M21" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N21" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O21" s="26" t="inlineStr">
@@ -4007,12 +4007,12 @@
       </c>
       <c r="N23" s="27" t="inlineStr">
         <is>
-          <t>abiFilters armeabi-v7a · operación Diego</t>
+          <t>COD-08-HU06-tuu-kozen/capturas/TC-RG-01*; 07_Plan_de_Pruebas/05_Evidencias_por_sprint/Sprint_03/capturas_20261013/; jest-hu06Tuu-factory-deteccion-output-20261011.txt</t>
         </is>
       </c>
       <c r="O23" s="26" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="P23" s="27" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="S23" s="27" t="inlineStr">
         <is>
-          <t>Alineado con el DAS (Kozen + TUU). Producción D-PAY 2.0 (Diego). Bloqueo solo de la regresión manual en QA Capstone.</t>
+          <t>Parcial 13/10/2026: Diego Madrid, Kozen P8 Neo. Débito $2.000 aprobado; crédito $5.000 cancelado (no declined emisor). Falta crédito aprobado. Jest 17/17 (11/10).</t>
         </is>
       </c>
     </row>
@@ -4166,12 +4166,12 @@
       </c>
       <c r="G25" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H25" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I25" s="26" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="K25" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L25" s="27" t="inlineStr">
@@ -4196,12 +4196,12 @@
       </c>
       <c r="M25" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N25" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O25" s="26" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="P25" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q25" s="27" t="inlineStr">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="K26" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L26" s="27" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="K28" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L28" s="27" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="K30" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L30" s="27" t="inlineStr">
@@ -4681,12 +4681,12 @@
       </c>
       <c r="M30" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N30" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O30" s="26" t="inlineStr">
@@ -4778,12 +4778,12 @@
       </c>
       <c r="M31" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N31" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O31" s="26" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="N32" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O32" s="26" t="inlineStr">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="K34" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L34" s="27" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="K35" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L35" s="27" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="K36" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L36" s="27" t="inlineStr">
@@ -6332,7 +6332,7 @@
     <row r="1" ht="30" customHeight="1" s="33">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>Escenarios de calidad (DAS §Vista de escenarios)</t>
+          <t>Escenarios de calidad (DAS ver Seccion Vista de escenarios)</t>
         </is>
       </c>
     </row>

</xml_diff>